<commit_message>
Add Ecoventure UI, groundwater reporting, and Windows deployment.
Ecoventure branding and layout refactor, groundwater profiles and samples,
Windows deploy launcher, Docker Compose, and team rollout documentation.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/phase1_251106R_data.xlsx
+++ b/samples/phase1_251106R_data.xlsx
@@ -909,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -932,100 +932,338 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>drilling_waste_intro</t>
+          <t>closure_recommendation</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>option_1_aer</t>
+          <t>support_closure</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Drilling waste was managed in accordance with AER requirements. Option 1 (AER, 2014) applies to this well.</t>
+          <t>Based on the data presented, Ecoventure supports proceeding with regulatory closure documentation, subject to agency review.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>drilling_waste_intro</t>
+          <t>closure_recommendation</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>option_2</t>
+          <t>defer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Drilling waste was managed under an approved alternative disposal pathway. Details are summarized in the drilling waste table.</t>
+          <t>Ecoventure recommends deferring closure until additional monitoring or remedial work is completed.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>phase2_recommendation</t>
+          <t>confirmatory_summary</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>recommended</t>
+          <t>met</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
+          <t>Confirmatory sampling results indicate that remedial objectives were met for the parameters and media evaluated.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>phase2_recommendation</t>
+          <t>confirmatory_summary</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>not_required</t>
+          <t>not_met</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is not recommended at this time, subject to client direction and future land use.</t>
+          <t>Confirmatory sampling results indicate that additional remedial action or monitoring is required for one or more parameters.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>site_recon_intro</t>
+          <t>drilling_waste_intro</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>not_completed</t>
+          <t>option_1_aer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+          <t>Drilling waste was managed in accordance with AER requirements. Option 1 (AER, 2014) applies to this well.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>drilling_waste_intro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>option_2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Drilling waste was managed under an approved alternative disposal pathway. Details are summarized in the drilling waste table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gw_data_usability</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>usable</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Field notes and laboratory quality control indicate that the groundwater data are suitable for comparison to applicable guidelines, subject to the limitations noted herein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>gw_data_usability</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>qualified</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Some data limitations are noted in the field log and tables below; interpreted trends should be considered qualified where purge volumes or hold times were atypical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>gw_program_intro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>This report presents results of the annual groundwater monitoring program conducted to assess groundwater quality and water levels relative to applicable Alberta guidelines and site-specific objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>gw_program_intro</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>This report summarizes baseline groundwater quality and static water levels following installation of the monitoring well network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>gw_recommendations</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ecoventure recommends continued groundwater monitoring at the established frequency to evaluate temporal trends and confirm stability of exceedances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>gw_recommendations</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ecoventure recommends additional investigation of exceedances identified in this reporting period, including potential source areas and downgradient wells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>gw_sampling_methods</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>low_flow</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Groundwater samples were collected using low-flow purging and sampling methods in accordance with project-specific sampling procedures and laboratory requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>gw_sampling_methods</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bailer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Groundwater samples were collected after purging each monitoring well until field parameters stabilized, using dedicated sampling equipment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>not_required</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is not recommended at this time, subject to client direction and future land use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>remediation_status</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Remediation activities are ongoing at the site under an approved remedial action plan. This report summarizes confirmatory sampling and progress toward remedial objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>remediation_status</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>confirmatory</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>This report documents confirmatory groundwater and soil sampling conducted to verify achievement of remedial objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>site_recon_intro</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>not_completed</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>A site visit was completed as part of this Phase I ESA. Observations from the visit are summarized below and in the site visit checklist.</t>
         </is>

</xml_diff>

<commit_message>
Align Phase I Alberta workflow with AER SED 002 Section 10 and improve render performance.
Add SED 002 checklist, compliance preflight, Phase II decision heuristics, OneStop export bundle, Devon sample pair, and faster single-pass template/Excel parsing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/phase1_251106R_data.xlsx
+++ b/samples/phase1_251106R_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ2"/>
+  <dimension ref="A1:AS2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,135 +467,180 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>asset_activity_type</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>prior_reclamation_cert_number</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>site_visit_date</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>records_review_summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>interview_operator_summary</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>interview_landowner_summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>flare_pit_used</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>no_drilling_waste_on_site</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>site_visit_photo_notes</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>qp_names</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>spud_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>cased_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>final_drill_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>well_depth_m</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>well_status</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>reentry</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>reentry_detail</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>production_fluid</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>aer_waste_compliance_option</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>drilling_waste_summary</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>phase2_drilling_waste_required</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>phase2_esa_required</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>client_phase_keyword</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>site_visit_completed</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>air_photo_observations</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>investigations_recommended</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>infrastructure_summary</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>spills_releases</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>conclusions_recommendations</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>drilling_waste_intro_selected</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>site_recon_intro_selected</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>phase2_recommendation_selected</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>executive_summary</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>drilling_waste_intro</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>site_recon_intro</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>phase2_recommendation</t>
         </is>
@@ -649,118 +694,147 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>Oil well site — drilled and abandoned / suspended</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Company well file, AER spills search, ABADATA, and historical air photos reviewed.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Informational interview with former site operator regarding waste disposal and infrastructure.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>Ecoventure QP (P.Eng.); Ecoventure QP (R.T.Ag.)</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>15-Mar-2004</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>17-Mar-2004</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>19-Jun-2004</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="W2" t="n">
         <v>710</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>suspended</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>The well was re-entered in June 2004 and drilled to a total depth of 710 metres (m), and the well is currently suspended</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>gas with water</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Option 1 (AER, 2014)</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>110 m3 of drilling waste (surface mud and fasthole mud) was disposed of via LWD at SW1/4 04-049-04 W4M, 35 m3 of mainhole drilling mud was landsprayed at SE-09-049-04 W4M, 3 m3 of shale was landspread onsite, and 60 m3 of mainhole drilling mud was hauled to the remote site at Example 10-04-048-06 W4M</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Phase II</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>The 2015 historical air photo shows the well centre and a possible disturbance area southeast of well centre for the containment berm and tanks</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>well centre and the production areas be investigated</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Access road, teardrop, wellhead, containment berm for production tanks</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Investigate well centre and production areas. Phase II ESA recommended.</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>option_1_aer</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>not_completed</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>recommended</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>Ecoventure Inc. was contracted by Base Element Energy Inc. to conduct a Phase I Environmental Site Assessment on the wellsite and associated facilities known as 15-20-049-10 W5M.  The well was spud 15-Mar-2004 and cased on 17-Mar-2004.  The well was re-entered in June 2004 and drilled to a total depth of 710 metres (m), and the well is currently suspended.  The well produced gas with water.
 The drilling waste was assessed using Checklist Compliance Option 1 (AER, 2014); 110 m3 of drilling waste (surface mud and fasthole mud) was disposed of via LWD at SW1/4 04-049-04 W4M, 35 m3 of mainhole drilling mud was landsprayed at SE-09-049-04 W4M, 3 m3 of shale was landspread onsite, and 60 m3 of mainhole drilling mud was hauled to the remote site at Example 10-04-048-06 W4M.
@@ -768,17 +842,17 @@
 After reviewing regulatory information and records, and conducting informational interviews; it is recommended that well centre and the production areas be investigated. The Base Element Energy Inc. keyword is Phase II.</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Drilling waste was managed in accordance with AER requirements. Option 1 (AER, 2014) applies to this well.</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
         </is>
@@ -795,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,6 +893,36 @@
           <t>location</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>disposal_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>gps_coordinates</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sump_depth_m</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cover_depth_m</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>remote_cert_number</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>waste_manifest_refs</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -839,6 +943,16 @@
           <t>SW1/4 04-049-04 W4M; SE-09-049-04 W4M; onsite; remote site</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>off-lease and on-lease</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Prepare Streamlit Community Cloud tester deploy.
Hosted mode reads Cloud secrets, remove localhost serverAddress, ship help/UX polish and platform modules needed for share.streamlit.io.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/phase1_251106R_data.xlsx
+++ b/samples/phase1_251106R_data.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DrillingWaste" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DwdaChecklist" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StorageTanks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhraseCatalog" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apecs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhraseCatalog" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1319,6 +1320,157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>apec_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>apec_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>location_description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>concern_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>source_of_concern</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>evidence_summary</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_document</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>phase2_recommended</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>APEC-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Historical flare pit</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SW corner of lease</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>flare_pit</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>air_photo</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Air photos show former flare pit depression.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>appendix_c_air_photos.pdf</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Sample for confirmation if Phase II proceeds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>APEC-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Produced water tank berm</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SE of well centre</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>storage_tank</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>records</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Above-ground produced water tank noted in records.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>historical_phase1.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>